<commit_message>
interim checking -- verification of square45-90 hough
</commit_message>
<xml_diff>
--- a/src/square45-90_sobel_exp.bin.hough.xlsx
+++ b/src/square45-90_sobel_exp.bin.hough.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kushn\Dropbox\software\projects\cv\cv-workbench\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{370F70E1-A501-4CAD-8C9F-A515D9C31AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0974AE2F-94AB-4DD0-A145-2C40C2E58371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="-50" yWindow="50" windowWidth="9280" windowHeight="9380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="square45-90_sobel_exp.bin.hough" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,19 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'square45-90_sobel_exp.bin.hough'!$A$1:$Z$19</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -621,7 +633,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>30</xdr:col>
-      <xdr:colOff>206010</xdr:colOff>
+      <xdr:colOff>183598</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>135870</xdr:rowOff>
     </xdr:to>
@@ -960,17 +972,17 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Z19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="8" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="15" width="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="26" width="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="8" width="6.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="5.90625" bestFit="1" customWidth="1"/>
+    <col min="12" max="15" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.90625" bestFit="1" customWidth="1"/>
+    <col min="17" max="26" width="6.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.35">
       <c r="B1">
         <v>-158.5</v>
       </c>
@@ -1047,7 +1059,7 @@
         <v>462.5</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1127,7 +1139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>3</v>
       </c>
@@ -1207,7 +1219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>6</v>
       </c>
@@ -1287,7 +1299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>9</v>
       </c>
@@ -1367,7 +1379,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>12</v>
       </c>
@@ -1447,7 +1459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>36</v>
       </c>
@@ -1527,7 +1539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>39</v>
       </c>
@@ -1607,7 +1619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>42</v>
       </c>
@@ -1687,7 +1699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>45</v>
       </c>
@@ -1767,7 +1779,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>48</v>
       </c>
@@ -1847,7 +1859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>51</v>
       </c>
@@ -1927,7 +1939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>54</v>
       </c>
@@ -2007,7 +2019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>129</v>
       </c>
@@ -2087,7 +2099,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>132</v>
       </c>
@@ -2167,7 +2179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>135</v>
       </c>
@@ -2247,7 +2259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>138</v>
       </c>
@@ -2327,7 +2339,7 @@
         <v>3373</v>
       </c>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>174</v>
       </c>
@@ -2407,7 +2419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>177</v>
       </c>

</xml_diff>